<commit_message>
Let each trip keep its charge, room, and food, and raise the hotel when the group needs another room.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/content/safar-electrified.xlsx
+++ b/content/safar-electrified.xlsx
@@ -91,7 +91,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -113,11 +113,25 @@
         <color rgb="00E3DDD0"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D3C7"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D3C7"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D3C7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D3C7"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -139,6 +153,10 @@
     </xf>
     <xf numFmtId="164" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -546,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -560,6 +578,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -660,7 +679,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="96" customHeight="1">
+    <row r="11" ht="120" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Costs — basis</t>
@@ -668,10 +687,10 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>trip = poori gaadi ka bill (charging, toll). Room badhta nahi, log badhte hain to ye split hota hai.
+          <t>trip = poori gaadi ka bill (charging, toll). Log badhenge to ye split hota hai, amount nahi badhta.
 person = har insaan pe ek baar.
 person_day = khana. Yahi amount food slider ki shuruaat hai (per person per day).
-room_night = hotel. 2 log = 1 room. Log badhenge to room badhega.</t>
+room_night = ek room ki ek raat ki keemat. Trips sheet me per_room likho — ek room me kitne log. 3 likha aur group 5 ya 6 hua to 2 room banenge aur hotel ka bill badhega. Khali chhodo to 2 log ek room. Alag hotel pe alag limit ho to Costs sheet ke per_room me likho.</t>
         </is>
       </c>
     </row>
@@ -720,6 +739,18 @@
       <c r="B15" s="4" t="inlineStr">
         <is>
           <t>Key column mat badalna. Sirf value column edit karo — headline, about, YouTube, Instagram, WhatsApp, UPI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="72" customHeight="1">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>Checkpoints aur paisa</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Stops sheet me har stop ka naam, kind (charge, food, stay), notes, aur amount. Amount us stop pe laga hua paisa hai — charge ka bill, khana, ya room. Film ke neeche ye list khulti hai. Tap karo to note aur rupaye khulte hain.</t>
         </is>
       </c>
     </row>
@@ -886,7 +917,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:R3"/>
+  <dimension ref="A1:S3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -906,6 +937,7 @@
     <col width="32" customWidth="1" min="15" max="15"/>
     <col width="42" customWidth="1" min="16" max="16"/>
     <col width="70" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -997,6 +1029,11 @@
       <c r="R1" t="inlineStr">
         <is>
           <t>status</t>
+        </is>
+      </c>
+      <c r="S1" s="11" t="inlineStr">
+        <is>
+          <t>per_room</t>
         </is>
       </c>
     </row>
@@ -1128,7 +1165,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1139,6 +1176,7 @@
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="55" customWidth="1" min="7" max="7"/>
     <col width="36" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1180,6 +1218,11 @@
       <c r="H1" s="5" t="inlineStr">
         <is>
           <t>photo_url</t>
+        </is>
+      </c>
+      <c r="I1" s="11" t="inlineStr">
+        <is>
+          <t>amount</t>
         </is>
       </c>
     </row>
@@ -1206,7 +1249,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1216,6 +1259,7 @@
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="55" customWidth="1" min="6" max="6"/>
     <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1252,6 +1296,11 @@
       <c r="G1" s="5" t="inlineStr">
         <is>
           <t>proof_url</t>
+        </is>
+      </c>
+      <c r="H1" s="11" t="inlineStr">
+        <is>
+          <t>per_room</t>
         </is>
       </c>
     </row>

</xml_diff>